<commit_message>
Inclusão scipt de substituição de IRF
</commit_message>
<xml_diff>
--- a/Planilhas/Fornecedores.xlsx
+++ b/Planilhas/Fornecedores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="EstaPastaDeTrabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ronaldo.gontijo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D3F2390-AF0F-4909-9389-D41C24C6734F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38EFF441-A4C8-4548-A261-590FF7AC0FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnvioNotas" sheetId="1" r:id="rId1"/>
@@ -20,169 +20,302 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
   <si>
     <t>LIFNR</t>
   </si>
   <si>
-    <t>0001001199</t>
-  </si>
-  <si>
-    <t>0001001211</t>
-  </si>
-  <si>
-    <t>0001001230</t>
-  </si>
-  <si>
-    <t>0001001232</t>
-  </si>
-  <si>
-    <t>0001001243</t>
-  </si>
-  <si>
-    <t>0001001246</t>
-  </si>
-  <si>
-    <t>0001001254</t>
-  </si>
-  <si>
-    <t>0001001255</t>
-  </si>
-  <si>
-    <t>0001001282</t>
-  </si>
-  <si>
-    <t>0001001283</t>
-  </si>
-  <si>
-    <t>0001001284</t>
-  </si>
-  <si>
-    <t>0001001287</t>
-  </si>
-  <si>
-    <t>0001001294</t>
-  </si>
-  <si>
-    <t>0001001328</t>
-  </si>
-  <si>
-    <t>0001001340</t>
-  </si>
-  <si>
-    <t>0001001358</t>
-  </si>
-  <si>
-    <t>0001001364</t>
-  </si>
-  <si>
-    <t>0001001369</t>
-  </si>
-  <si>
-    <t>0001001375</t>
-  </si>
-  <si>
-    <t>0001001379</t>
-  </si>
-  <si>
-    <t>0001001388</t>
-  </si>
-  <si>
-    <t>0001001394</t>
-  </si>
-  <si>
-    <t>0001001403</t>
-  </si>
-  <si>
-    <t>0001001502</t>
-  </si>
-  <si>
-    <t>0001001516</t>
-  </si>
-  <si>
-    <t>0001001522</t>
-  </si>
-  <si>
-    <t>0001001527</t>
-  </si>
-  <si>
-    <t>0001001556</t>
-  </si>
-  <si>
-    <t>0001001557</t>
-  </si>
-  <si>
-    <t>0001001577</t>
-  </si>
-  <si>
-    <t>0001001580</t>
-  </si>
-  <si>
-    <t>0001001589</t>
-  </si>
-  <si>
-    <t>0001001597</t>
-  </si>
-  <si>
-    <t>0001001598</t>
-  </si>
-  <si>
-    <t>0001001605</t>
-  </si>
-  <si>
-    <t>0001001608</t>
-  </si>
-  <si>
-    <t>0001001610</t>
-  </si>
-  <si>
-    <t>0001001612</t>
-  </si>
-  <si>
-    <t>0001001631</t>
-  </si>
-  <si>
-    <t>0001001689</t>
-  </si>
-  <si>
-    <t>0001001713</t>
-  </si>
-  <si>
-    <t>0001001753</t>
-  </si>
-  <si>
-    <t>0001001759</t>
-  </si>
-  <si>
-    <t>0001001761</t>
-  </si>
-  <si>
-    <t>0001001768</t>
-  </si>
-  <si>
-    <t>0001001771</t>
-  </si>
-  <si>
-    <t>0001001781</t>
-  </si>
-  <si>
-    <t>0001001784</t>
-  </si>
-  <si>
-    <t>0001001785</t>
-  </si>
-  <si>
-    <t>0001001786</t>
+    <t>1003959</t>
+  </si>
+  <si>
+    <t>1003965</t>
+  </si>
+  <si>
+    <t>1003967</t>
+  </si>
+  <si>
+    <t>1003982</t>
+  </si>
+  <si>
+    <t>1003999</t>
+  </si>
+  <si>
+    <t>1004033</t>
+  </si>
+  <si>
+    <t>1004054</t>
+  </si>
+  <si>
+    <t>1004122</t>
+  </si>
+  <si>
+    <t>1004314</t>
+  </si>
+  <si>
+    <t>1004357</t>
+  </si>
+  <si>
+    <t>1004425</t>
+  </si>
+  <si>
+    <t>1004428</t>
+  </si>
+  <si>
+    <t>1004436</t>
+  </si>
+  <si>
+    <t>1004461</t>
+  </si>
+  <si>
+    <t>1004529</t>
+  </si>
+  <si>
+    <t>1004554</t>
+  </si>
+  <si>
+    <t>1004555</t>
+  </si>
+  <si>
+    <t>1004556</t>
+  </si>
+  <si>
+    <t>1004558</t>
+  </si>
+  <si>
+    <t>1004560</t>
+  </si>
+  <si>
+    <t>1004564</t>
+  </si>
+  <si>
+    <t>1004565</t>
+  </si>
+  <si>
+    <t>1004566</t>
+  </si>
+  <si>
+    <t>1004573</t>
+  </si>
+  <si>
+    <t>1004577</t>
+  </si>
+  <si>
+    <t>1004589</t>
+  </si>
+  <si>
+    <t>1004598</t>
+  </si>
+  <si>
+    <t>1004599</t>
+  </si>
+  <si>
+    <t>1004602</t>
+  </si>
+  <si>
+    <t>1004603</t>
+  </si>
+  <si>
+    <t>1004604</t>
+  </si>
+  <si>
+    <t>1004616</t>
+  </si>
+  <si>
+    <t>1004620</t>
+  </si>
+  <si>
+    <t>1004621</t>
+  </si>
+  <si>
+    <t>1004622</t>
+  </si>
+  <si>
+    <t>1004628</t>
+  </si>
+  <si>
+    <t>1004634</t>
+  </si>
+  <si>
+    <t>1004640</t>
+  </si>
+  <si>
+    <t>1004649</t>
+  </si>
+  <si>
+    <t>1004651</t>
+  </si>
+  <si>
+    <t>1004665</t>
+  </si>
+  <si>
+    <t>1004675</t>
+  </si>
+  <si>
+    <t>1004684</t>
+  </si>
+  <si>
+    <t>1004694</t>
+  </si>
+  <si>
+    <t>1004698</t>
+  </si>
+  <si>
+    <t>1004709</t>
+  </si>
+  <si>
+    <t>1004750</t>
+  </si>
+  <si>
+    <t>1004801</t>
+  </si>
+  <si>
+    <t>1004810</t>
+  </si>
+  <si>
+    <t>1004812</t>
+  </si>
+  <si>
+    <t>1004813</t>
+  </si>
+  <si>
+    <t>1029402</t>
+  </si>
+  <si>
+    <t>1029435</t>
+  </si>
+  <si>
+    <t>1029687</t>
+  </si>
+  <si>
+    <t>1029692</t>
+  </si>
+  <si>
+    <t>1029693</t>
+  </si>
+  <si>
+    <t>1030724</t>
+  </si>
+  <si>
+    <t>1031013</t>
+  </si>
+  <si>
+    <t>1031150</t>
+  </si>
+  <si>
+    <t>1031219</t>
+  </si>
+  <si>
+    <t>1031312</t>
+  </si>
+  <si>
+    <t>1031363</t>
+  </si>
+  <si>
+    <t>1031427</t>
+  </si>
+  <si>
+    <t>1031573</t>
+  </si>
+  <si>
+    <t>1031589</t>
+  </si>
+  <si>
+    <t>1031592</t>
+  </si>
+  <si>
+    <t>1031629</t>
+  </si>
+  <si>
+    <t>1031772</t>
+  </si>
+  <si>
+    <t>1031795</t>
+  </si>
+  <si>
+    <t>1031910</t>
+  </si>
+  <si>
+    <t>1031942</t>
+  </si>
+  <si>
+    <t>1031969</t>
+  </si>
+  <si>
+    <t>1032075</t>
+  </si>
+  <si>
+    <t>1032137</t>
+  </si>
+  <si>
+    <t>1032138</t>
+  </si>
+  <si>
+    <t>1032168</t>
+  </si>
+  <si>
+    <t>1032172</t>
+  </si>
+  <si>
+    <t>1032249</t>
+  </si>
+  <si>
+    <t>1032448</t>
+  </si>
+  <si>
+    <t>1032667</t>
+  </si>
+  <si>
+    <t>1032675</t>
+  </si>
+  <si>
+    <t>1032676</t>
+  </si>
+  <si>
+    <t>1032677</t>
+  </si>
+  <si>
+    <t>1032678</t>
+  </si>
+  <si>
+    <t>1032680</t>
+  </si>
+  <si>
+    <t>1032681</t>
+  </si>
+  <si>
+    <t>1032800</t>
+  </si>
+  <si>
+    <t>1032801</t>
+  </si>
+  <si>
+    <t>1032828</t>
+  </si>
+  <si>
+    <t>1032833</t>
+  </si>
+  <si>
+    <t>1032885</t>
+  </si>
+  <si>
+    <t>1032922</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -208,16 +341,57 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -235,10 +409,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela1" displayName="Tabela1" ref="A1:A51" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:A51" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela1" displayName="Tabela1" ref="A1:A94" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1">
+  <autoFilter ref="A1:A94" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="LIFNR"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="LIFNR" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -530,7 +704,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -552,253 +726,468 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+      <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="A34" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+      <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+      <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+      <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+      <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+      <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+      <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+      <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+      <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+      <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+      <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+      <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+      <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+      <c r="A50" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+      <c r="A51" s="2" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" s="2">
+        <v>1032619</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A84" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" s="2" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>